<commit_message>
Add Wandering Merchant UR resource choice chest
</commit_message>
<xml_diff>
--- a/data/Last War Price Guide.xlsx
+++ b/data/Last War Price Guide.xlsx
@@ -1369,6 +1369,22 @@
       <c r="BS4" t="n">
         <v>10</v>
       </c>
+      <c r="BU4" t="inlineStr">
+        <is>
+          <t>Resource Choice Chest (UR)</t>
+        </is>
+      </c>
+      <c r="BV4" t="n">
+        <v>10</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="BX4" t="inlineStr">
+        <is>
+          <t>DIA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
Add Honor Store weapon shard and stamina
</commit_message>
<xml_diff>
--- a/data/Last War Price Guide.xlsx
+++ b/data/Last War Price Guide.xlsx
@@ -2846,6 +2846,25 @@
       <c r="Q12" t="n">
         <v>3</v>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Universal Exclusive Weapon Shard</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>1</v>
+      </c>
+      <c r="U12" t="n">
+        <v>2500</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="W12" t="n">
+        <v>25</v>
+      </c>
       <c r="Y12" t="inlineStr">
         <is>
           <t>Drone Parts</t>
@@ -2996,6 +3015,25 @@
       </c>
       <c r="Q13" t="n">
         <v>3</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Stamina</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>50</v>
+      </c>
+      <c r="U13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="W13" t="n">
+        <v>50</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Serum Shop for Season 1
</commit_message>
<xml_diff>
--- a/data/Last War Price Guide.xlsx
+++ b/data/Last War Price Guide.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BY28"/>
+  <dimension ref="A1:CE28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -486,6 +486,11 @@
     <col width="13" customWidth="1" min="75" max="75"/>
     <col width="13" customWidth="1" min="76" max="76"/>
     <col width="13" customWidth="1" min="77" max="77"/>
+    <col width="29.77734375" customWidth="1" min="79" max="79"/>
+    <col width="13" customWidth="1" min="80" max="80"/>
+    <col width="13" customWidth="1" min="81" max="81"/>
+    <col width="13" customWidth="1" min="82" max="82"/>
+    <col width="13" customWidth="1" min="83" max="83"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -571,6 +576,11 @@
           <t>Wandering Merchant</t>
         </is>
       </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>Serum Shop</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -899,6 +909,31 @@
           <t>Limit</t>
         </is>
       </c>
+      <c r="CA2" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="CB2" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="CC2" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="CD2" s="1" t="inlineStr">
+        <is>
+          <t>Curr</t>
+        </is>
+      </c>
+      <c r="CE2" s="1" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1142,6 +1177,25 @@
           <t>DIA</t>
         </is>
       </c>
+      <c r="CA3" t="inlineStr">
+        <is>
+          <t>UR Hero Universal Shard</t>
+        </is>
+      </c>
+      <c r="CB3" t="n">
+        <v>10</v>
+      </c>
+      <c r="CC3" t="n">
+        <v>100</v>
+      </c>
+      <c r="CD3" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1385,6 +1439,22 @@
           <t>DIA</t>
         </is>
       </c>
+      <c r="CA4" t="inlineStr">
+        <is>
+          <t>Drone Parts</t>
+        </is>
+      </c>
+      <c r="CB4" t="n">
+        <v>20</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>100</v>
+      </c>
+      <c r="CD4" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1612,6 +1682,22 @@
       <c r="BS5" t="n">
         <v>1</v>
       </c>
+      <c r="CA5" t="inlineStr">
+        <is>
+          <t>S1 Skill Point</t>
+        </is>
+      </c>
+      <c r="CB5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>100</v>
+      </c>
+      <c r="CD5" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1839,6 +1925,22 @@
       <c r="BS6" t="n">
         <v>10</v>
       </c>
+      <c r="CA6" t="inlineStr">
+        <is>
+          <t>Universal Exclusive Weapon Shard</t>
+        </is>
+      </c>
+      <c r="CB6" t="n">
+        <v>10</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>100</v>
+      </c>
+      <c r="CD6" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2066,6 +2168,25 @@
       <c r="BS7" t="n">
         <v>10</v>
       </c>
+      <c r="CA7" t="inlineStr">
+        <is>
+          <t>Recruitment Orders</t>
+        </is>
+      </c>
+      <c r="CB7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>500</v>
+      </c>
+      <c r="CD7" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2255,6 +2376,25 @@
       <c r="BS8" t="n">
         <v>10</v>
       </c>
+      <c r="CA8" t="inlineStr">
+        <is>
+          <t>Profession EXP</t>
+        </is>
+      </c>
+      <c r="CB8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>20</v>
+      </c>
+      <c r="CD8" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE8" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2444,6 +2584,25 @@
       <c r="BS9" t="n">
         <v>10</v>
       </c>
+      <c r="CA9" t="inlineStr">
+        <is>
+          <t>Mutant Crystals</t>
+        </is>
+      </c>
+      <c r="CB9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>10</v>
+      </c>
+      <c r="CD9" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE9" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2633,6 +2792,25 @@
       <c r="BS10" t="n">
         <v>10</v>
       </c>
+      <c r="CA10" t="inlineStr">
+        <is>
+          <t>Iron Chest (SSR)</t>
+        </is>
+      </c>
+      <c r="CB10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>20</v>
+      </c>
+      <c r="CD10" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE10" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="11">
       <c r="G11" t="inlineStr">
@@ -2806,6 +2984,25 @@
       <c r="BS11" t="n">
         <v>10</v>
       </c>
+      <c r="CA11" t="inlineStr">
+        <is>
+          <t>Coin Chest (SSR)</t>
+        </is>
+      </c>
+      <c r="CB11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>20</v>
+      </c>
+      <c r="CD11" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE11" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="12">
       <c r="G12" t="inlineStr">
@@ -2976,6 +3173,25 @@
       <c r="BS12" t="n">
         <v>10</v>
       </c>
+      <c r="CA12" t="inlineStr">
+        <is>
+          <t>Food Chest (SSR)</t>
+        </is>
+      </c>
+      <c r="CB12" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>20</v>
+      </c>
+      <c r="CD12" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE12" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="13">
       <c r="G13" t="inlineStr">
@@ -3130,6 +3346,25 @@
       <c r="BS13" t="n">
         <v>10</v>
       </c>
+      <c r="CA13" t="inlineStr">
+        <is>
+          <t>5m Construction Speed-Up</t>
+        </is>
+      </c>
+      <c r="CB13" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC13" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD13" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE13" t="n">
+        <v>9999</v>
+      </c>
     </row>
     <row r="14">
       <c r="G14" t="inlineStr">
@@ -3224,6 +3459,25 @@
       <c r="BG14" t="n">
         <v>1000</v>
       </c>
+      <c r="CA14" t="inlineStr">
+        <is>
+          <t>5m Research Speed-Up</t>
+        </is>
+      </c>
+      <c r="CB14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD14" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE14" t="n">
+        <v>9999</v>
+      </c>
     </row>
     <row r="15">
       <c r="G15" t="inlineStr">
@@ -3317,6 +3571,25 @@
       </c>
       <c r="BG15" t="n">
         <v>200</v>
+      </c>
+      <c r="CA15" t="inlineStr">
+        <is>
+          <t>5m Training Speed-Up</t>
+        </is>
+      </c>
+      <c r="CB15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD15" t="inlineStr">
+        <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CE15" t="n">
+        <v>9999</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Add Season Storefront for Season 1
</commit_message>
<xml_diff>
--- a/data/Last War Price Guide.xlsx
+++ b/data/Last War Price Guide.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE28"/>
+  <dimension ref="A1:CK28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -491,6 +491,11 @@
     <col width="13" customWidth="1" min="81" max="81"/>
     <col width="13" customWidth="1" min="82" max="82"/>
     <col width="13" customWidth="1" min="83" max="83"/>
+    <col width="29.77734375" customWidth="1" min="85" max="85"/>
+    <col width="13" customWidth="1" min="86" max="86"/>
+    <col width="13" customWidth="1" min="87" max="87"/>
+    <col width="13" customWidth="1" min="88" max="88"/>
+    <col width="13" customWidth="1" min="89" max="89"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -581,6 +586,11 @@
           <t>Serum Shop</t>
         </is>
       </c>
+      <c r="CG1" t="inlineStr">
+        <is>
+          <t>Season Storefront</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -934,6 +944,31 @@
           <t>Limit</t>
         </is>
       </c>
+      <c r="CG2" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="CH2" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="CI2" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="CJ2" s="1" t="inlineStr">
+        <is>
+          <t>Curr</t>
+        </is>
+      </c>
+      <c r="CK2" s="1" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1196,6 +1231,25 @@
       <c r="CE3" t="n">
         <v>1</v>
       </c>
+      <c r="CG3" t="inlineStr">
+        <is>
+          <t>Dominance Sanctuary (Permanent)</t>
+        </is>
+      </c>
+      <c r="CH3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="CJ3" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="CK3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1455,6 +1509,25 @@
           <t>SER</t>
         </is>
       </c>
+      <c r="CG4" t="inlineStr">
+        <is>
+          <t>Gear Blueprint (MR)</t>
+        </is>
+      </c>
+      <c r="CH4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>100</v>
+      </c>
+      <c r="CJ4" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="CK4" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1698,6 +1771,25 @@
           <t>SER</t>
         </is>
       </c>
+      <c r="CG5" t="inlineStr">
+        <is>
+          <t>God of Judgment</t>
+        </is>
+      </c>
+      <c r="CH5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>80</v>
+      </c>
+      <c r="CJ5" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="CK5" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1941,6 +2033,25 @@
           <t>SER</t>
         </is>
       </c>
+      <c r="CG6" t="inlineStr">
+        <is>
+          <t>S1 Skill Point</t>
+        </is>
+      </c>
+      <c r="CH6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>50</v>
+      </c>
+      <c r="CJ6" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="CK6" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2187,6 +2298,25 @@
       <c r="CE7" t="n">
         <v>1</v>
       </c>
+      <c r="CG7" t="inlineStr">
+        <is>
+          <t>Profession Change Certificate</t>
+        </is>
+      </c>
+      <c r="CH7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>50</v>
+      </c>
+      <c r="CJ7" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="CK7" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2395,6 +2525,25 @@
       <c r="CE8" t="n">
         <v>20</v>
       </c>
+      <c r="CG8" t="inlineStr">
+        <is>
+          <t>Profession Skill Reset Book</t>
+        </is>
+      </c>
+      <c r="CH8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>10</v>
+      </c>
+      <c r="CJ8" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="CK8" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2603,6 +2752,25 @@
       <c r="CE9" t="n">
         <v>50</v>
       </c>
+      <c r="CG9" t="inlineStr">
+        <is>
+          <t>Sandstorm Master (Permanent)</t>
+        </is>
+      </c>
+      <c r="CH9" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>200</v>
+      </c>
+      <c r="CJ9" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="CK9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2810,6 +2978,25 @@
       </c>
       <c r="CE10" t="n">
         <v>100</v>
+      </c>
+      <c r="CG10" t="inlineStr">
+        <is>
+          <t>UR Hero Badge</t>
+        </is>
+      </c>
+      <c r="CH10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>50</v>
+      </c>
+      <c r="CJ10" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="CK10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Add VIP dielectric ceramic listing
</commit_message>
<xml_diff>
--- a/data/Last War Price Guide.xlsx
+++ b/data/Last War Price Guide.xlsx
@@ -4254,6 +4254,25 @@
       </c>
     </row>
     <row r="25">
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Dielectric Ceramic</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>64</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>DIA</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>50</v>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>1h Research Speed-Up</t>

</xml_diff>

<commit_message>
Add Zombie Invasion item limits
</commit_message>
<xml_diff>
--- a/data/Last War Price Guide.xlsx
+++ b/data/Last War Price Guide.xlsx
@@ -3284,6 +3284,9 @@
           <t>COUR</t>
         </is>
       </c>
+      <c r="AU12" t="n">
+        <v>3</v>
+      </c>
       <c r="AW12" t="inlineStr">
         <is>
           <t>Drone Parts</t>
@@ -3627,6 +3630,9 @@
           <t>COUR</t>
         </is>
       </c>
+      <c r="AU14" t="n">
+        <v>100</v>
+      </c>
       <c r="BC14" t="inlineStr">
         <is>
           <t>Resource Choice Chest (SSR)</t>
@@ -3739,6 +3745,9 @@
         <is>
           <t>COUR</t>
         </is>
+      </c>
+      <c r="AU15" t="n">
+        <v>50</v>
       </c>
       <c r="BC15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Bounty Hunter event limits
</commit_message>
<xml_diff>
--- a/data/Last War Price Guide.xlsx
+++ b/data/Last War Price Guide.xlsx
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="BA4" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="BC4" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="BA5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="BC5" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="BA9" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="BC9" t="inlineStr">
         <is>
@@ -2901,7 +2901,7 @@
         </is>
       </c>
       <c r="BA10" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="BC10" t="inlineStr">
         <is>
@@ -3112,7 +3112,7 @@
         </is>
       </c>
       <c r="BA11" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="BC11" t="inlineStr">
         <is>
@@ -3304,7 +3304,7 @@
         </is>
       </c>
       <c r="BA12" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="BC12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Gear Boost Choice Chest network source
</commit_message>
<xml_diff>
--- a/data/Last War Price Guide.xlsx
+++ b/data/Last War Price Guide.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CK28"/>
+  <dimension ref="A1:CQ28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.5546875" customWidth="1" min="1" max="1"/>
@@ -553,40 +553,45 @@
       </c>
       <c r="AQ1" t="inlineStr">
         <is>
+          <t>Gear Boost Choice Chest</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
           <t>Zombie Invasion Store</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>Bounty Hunter Trade Store</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>Glittering Market</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>Total Mobilization Store</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>ID Points Mall</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>Wandering Merchant</t>
         </is>
       </c>
-      <c r="CA1" t="inlineStr">
+      <c r="CG1" t="inlineStr">
         <is>
           <t>Serum Shop</t>
         </is>
       </c>
-      <c r="CG1" t="inlineStr">
+      <c r="CM1" t="inlineStr">
         <is>
           <t>Season Storefront</t>
         </is>
@@ -769,27 +774,27 @@
           <t>Limit</t>
         </is>
       </c>
-      <c r="AQ2" s="1" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="AR2" s="1" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="AS2" s="1" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="AT2" s="1" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>Curr</t>
         </is>
       </c>
-      <c r="AU2" s="1" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>Limit</t>
         </is>
@@ -965,6 +970,31 @@
         </is>
       </c>
       <c r="CK2" s="1" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="CM2" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="CN2" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="CO2" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="CP2" s="1" t="inlineStr">
+        <is>
+          <t>Curr</t>
+        </is>
+      </c>
+      <c r="CQ2" s="1" t="inlineStr">
         <is>
           <t>Limit</t>
         </is>
@@ -1103,26 +1133,26 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
+          <t>Gear Blueprint (UR)</t>
+        </is>
+      </c>
+      <c r="AR3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>GBC</t>
+        </is>
+      </c>
+      <c r="AU3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
           <t>Survivor Recruitment Ticket</t>
-        </is>
-      </c>
-      <c r="AR3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>80</v>
-      </c>
-      <c r="AT3" t="inlineStr">
-        <is>
-          <t>COUR</t>
-        </is>
-      </c>
-      <c r="AU3" t="n">
-        <v>30</v>
-      </c>
-      <c r="AW3" t="inlineStr">
-        <is>
-          <t>Lv 5 Drone Component Chest</t>
         </is>
       </c>
       <c r="AX3" t="n">
@@ -1133,121 +1163,140 @@
       </c>
       <c r="AZ3" t="inlineStr">
         <is>
+          <t>COUR</t>
+        </is>
+      </c>
+      <c r="BA3" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>Lv 5 Drone Component Chest</t>
+        </is>
+      </c>
+      <c r="BD3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>80</v>
+      </c>
+      <c r="BF3" t="inlineStr">
+        <is>
           <t>BOUN</t>
         </is>
       </c>
-      <c r="BA3" t="n">
+      <c r="BG3" t="n">
         <v>5</v>
       </c>
-      <c r="BC3" t="inlineStr">
+      <c r="BI3" t="inlineStr">
         <is>
           <t>Hero Choice Chest</t>
         </is>
       </c>
-      <c r="BD3" t="n">
-        <v>10</v>
-      </c>
-      <c r="BE3" t="n">
+      <c r="BJ3" t="n">
+        <v>10</v>
+      </c>
+      <c r="BK3" t="n">
         <v>60</v>
       </c>
-      <c r="BF3" t="inlineStr">
+      <c r="BL3" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI3" t="inlineStr">
+      <c r="BM3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO3" t="inlineStr">
         <is>
           <t>UR Hero Universal Shard</t>
         </is>
       </c>
-      <c r="BJ3" t="n">
-        <v>10</v>
-      </c>
-      <c r="BK3" t="n">
-        <v>10</v>
-      </c>
-      <c r="BL3" t="inlineStr">
+      <c r="BP3" t="n">
+        <v>10</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>10</v>
+      </c>
+      <c r="BR3" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BO3" t="inlineStr">
+      <c r="BS3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU3" t="inlineStr">
         <is>
           <t>UR Hero Universal Shard</t>
         </is>
       </c>
-      <c r="BP3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ3" t="n">
+      <c r="BV3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW3" t="n">
         <v>40</v>
       </c>
-      <c r="BR3" t="inlineStr">
+      <c r="BX3" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS3" t="n">
-        <v>10</v>
-      </c>
-      <c r="BU3" t="inlineStr">
+      <c r="BY3" t="n">
+        <v>10</v>
+      </c>
+      <c r="CA3" t="inlineStr">
         <is>
           <t>UR Hero Universal Shard</t>
         </is>
       </c>
-      <c r="BV3" t="n">
-        <v>10</v>
-      </c>
-      <c r="BW3" t="n">
+      <c r="CB3" t="n">
+        <v>10</v>
+      </c>
+      <c r="CC3" t="n">
         <v>2000</v>
       </c>
-      <c r="BX3" t="inlineStr">
+      <c r="CD3" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="CA3" t="inlineStr">
+      <c r="CG3" t="inlineStr">
         <is>
           <t>UR Hero Universal Shard</t>
         </is>
       </c>
-      <c r="CB3" t="n">
-        <v>10</v>
-      </c>
-      <c r="CC3" t="n">
+      <c r="CH3" t="n">
+        <v>10</v>
+      </c>
+      <c r="CI3" t="n">
         <v>100</v>
       </c>
-      <c r="CD3" t="inlineStr">
+      <c r="CJ3" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE3" t="n">
-        <v>1</v>
-      </c>
-      <c r="CG3" t="inlineStr">
+      <c r="CK3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM3" t="inlineStr">
         <is>
           <t>Dominance Sanctuary (Permanent)</t>
         </is>
       </c>
-      <c r="CH3" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI3" t="n">
+      <c r="CN3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO3" t="n">
         <v>1000</v>
       </c>
-      <c r="CJ3" t="inlineStr">
+      <c r="CP3" t="inlineStr">
         <is>
           <t>SEA</t>
         </is>
       </c>
-      <c r="CK3" t="n">
+      <c r="CQ3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1384,148 +1433,167 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
+          <t>Dielectric Ceramic</t>
+        </is>
+      </c>
+      <c r="AR4" t="n">
+        <v>100</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>GBC</t>
+        </is>
+      </c>
+      <c r="AU4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
           <t>SSR Iron Chest</t>
         </is>
       </c>
-      <c r="AR4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS4" t="n">
+      <c r="AX4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY4" t="n">
         <v>160</v>
       </c>
-      <c r="AT4" t="inlineStr">
+      <c r="AZ4" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU4" t="n">
+      <c r="BA4" t="n">
         <v>50</v>
       </c>
-      <c r="AW4" t="inlineStr">
+      <c r="BC4" t="inlineStr">
         <is>
           <t>Drone Parts</t>
         </is>
       </c>
-      <c r="AX4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AY4" t="n">
+      <c r="BD4" t="n">
+        <v>10</v>
+      </c>
+      <c r="BE4" t="n">
         <v>22</v>
       </c>
-      <c r="AZ4" t="inlineStr">
+      <c r="BF4" t="inlineStr">
         <is>
           <t>BOUN</t>
         </is>
       </c>
-      <c r="BA4" t="n">
+      <c r="BG4" t="n">
         <v>100</v>
       </c>
-      <c r="BC4" t="inlineStr">
+      <c r="BI4" t="inlineStr">
         <is>
           <t>Dielectric Ceramic</t>
         </is>
       </c>
-      <c r="BD4" t="n">
+      <c r="BJ4" t="n">
         <v>100</v>
       </c>
-      <c r="BE4" t="n">
+      <c r="BK4" t="n">
         <v>40</v>
       </c>
-      <c r="BF4" t="inlineStr">
+      <c r="BL4" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI4" t="inlineStr">
+      <c r="BM4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO4" t="inlineStr">
         <is>
           <t>Hero Choice Chest</t>
         </is>
       </c>
-      <c r="BJ4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK4" t="n">
+      <c r="BP4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ4" t="n">
         <v>2</v>
       </c>
-      <c r="BL4" t="inlineStr">
+      <c r="BR4" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM4" t="n">
+      <c r="BS4" t="n">
         <v>800</v>
       </c>
-      <c r="BO4" t="inlineStr">
+      <c r="BU4" t="inlineStr">
         <is>
           <t>Hero EXP Chest (SSR)</t>
         </is>
       </c>
-      <c r="BP4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ4" t="n">
+      <c r="BV4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW4" t="n">
         <v>20</v>
       </c>
-      <c r="BR4" t="inlineStr">
+      <c r="BX4" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS4" t="n">
-        <v>10</v>
-      </c>
-      <c r="BU4" t="inlineStr">
+      <c r="BY4" t="n">
+        <v>10</v>
+      </c>
+      <c r="CA4" t="inlineStr">
         <is>
           <t>Resource Choice Chest (UR)</t>
         </is>
       </c>
-      <c r="BV4" t="n">
-        <v>10</v>
-      </c>
-      <c r="BW4" t="n">
+      <c r="CB4" t="n">
+        <v>10</v>
+      </c>
+      <c r="CC4" t="n">
         <v>1500</v>
       </c>
-      <c r="BX4" t="inlineStr">
+      <c r="CD4" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="CA4" t="inlineStr">
+      <c r="CG4" t="inlineStr">
         <is>
           <t>Drone Parts</t>
         </is>
       </c>
-      <c r="CB4" t="n">
+      <c r="CH4" t="n">
         <v>20</v>
-      </c>
-      <c r="CC4" t="n">
-        <v>100</v>
-      </c>
-      <c r="CD4" t="inlineStr">
-        <is>
-          <t>SER</t>
-        </is>
-      </c>
-      <c r="CG4" t="inlineStr">
-        <is>
-          <t>Gear Blueprint (MR)</t>
-        </is>
-      </c>
-      <c r="CH4" t="n">
-        <v>1</v>
       </c>
       <c r="CI4" t="n">
         <v>100</v>
       </c>
       <c r="CJ4" t="inlineStr">
         <is>
+          <t>SER</t>
+        </is>
+      </c>
+      <c r="CM4" t="inlineStr">
+        <is>
+          <t>Gear Blueprint (MR)</t>
+        </is>
+      </c>
+      <c r="CN4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO4" t="n">
+        <v>100</v>
+      </c>
+      <c r="CP4" t="inlineStr">
+        <is>
           <t>SEA</t>
         </is>
       </c>
-      <c r="CK4" t="n">
+      <c r="CQ4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1662,132 +1730,151 @@
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
+          <t>Upgrade Ore</t>
+        </is>
+      </c>
+      <c r="AR5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>GBC</t>
+        </is>
+      </c>
+      <c r="AU5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
           <t>SSR Food Chest</t>
         </is>
       </c>
-      <c r="AR5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS5" t="n">
+      <c r="AX5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY5" t="n">
         <v>160</v>
       </c>
-      <c r="AT5" t="inlineStr">
+      <c r="AZ5" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU5" t="n">
+      <c r="BA5" t="n">
         <v>50</v>
       </c>
-      <c r="AW5" t="inlineStr">
+      <c r="BC5" t="inlineStr">
         <is>
           <t>Lv 5 Drone Component Choice Chest</t>
         </is>
       </c>
-      <c r="AX5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY5" t="n">
+      <c r="BD5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE5" t="n">
         <v>220</v>
       </c>
-      <c r="AZ5" t="inlineStr">
+      <c r="BF5" t="inlineStr">
         <is>
           <t>BOUN</t>
         </is>
       </c>
-      <c r="BA5" t="n">
-        <v>10</v>
-      </c>
-      <c r="BC5" t="inlineStr">
+      <c r="BG5" t="n">
+        <v>10</v>
+      </c>
+      <c r="BI5" t="inlineStr">
         <is>
           <t>Luxury Choice Chest</t>
         </is>
       </c>
-      <c r="BD5" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE5" t="n">
+      <c r="BJ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK5" t="n">
         <v>100</v>
       </c>
-      <c r="BF5" t="inlineStr">
+      <c r="BL5" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG5" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI5" t="inlineStr">
+      <c r="BM5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO5" t="inlineStr">
         <is>
           <t>Survivor Recruitment Ticket</t>
         </is>
       </c>
-      <c r="BJ5" t="n">
-        <v>10</v>
-      </c>
-      <c r="BK5" t="n">
+      <c r="BP5" t="n">
+        <v>10</v>
+      </c>
+      <c r="BQ5" t="n">
         <v>8</v>
       </c>
-      <c r="BL5" t="inlineStr">
+      <c r="BR5" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM5" t="n">
+      <c r="BS5" t="n">
         <v>50</v>
       </c>
-      <c r="BO5" t="inlineStr">
+      <c r="BU5" t="inlineStr">
         <is>
           <t>Emote (Gold Bricks)</t>
         </is>
       </c>
-      <c r="BP5" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ5" t="n">
+      <c r="BV5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW5" t="n">
         <v>100</v>
       </c>
-      <c r="BR5" t="inlineStr">
+      <c r="BX5" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS5" t="n">
-        <v>1</v>
-      </c>
-      <c r="CA5" t="inlineStr">
+      <c r="BY5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG5" t="inlineStr">
         <is>
           <t>S1 Skill Point</t>
         </is>
       </c>
-      <c r="CB5" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC5" t="n">
+      <c r="CH5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI5" t="n">
         <v>100</v>
       </c>
-      <c r="CD5" t="inlineStr">
+      <c r="CJ5" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CG5" t="inlineStr">
+      <c r="CM5" t="inlineStr">
         <is>
           <t>God of Judgment</t>
         </is>
       </c>
-      <c r="CH5" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI5" t="n">
+      <c r="CN5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO5" t="n">
         <v>80</v>
       </c>
-      <c r="CJ5" t="inlineStr">
+      <c r="CP5" t="inlineStr">
         <is>
           <t>SEA</t>
         </is>
       </c>
-      <c r="CK5" t="n">
+      <c r="CQ5" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1922,39 +2009,20 @@
       <c r="AO6" t="n">
         <v>1</v>
       </c>
-      <c r="AQ6" t="inlineStr">
+      <c r="AW6" t="inlineStr">
         <is>
           <t>SSR Coin Chest</t>
         </is>
       </c>
-      <c r="AR6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS6" t="n">
+      <c r="AX6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY6" t="n">
         <v>160</v>
       </c>
-      <c r="AT6" t="inlineStr">
+      <c r="AZ6" t="inlineStr">
         <is>
           <t>COUR</t>
-        </is>
-      </c>
-      <c r="AU6" t="n">
-        <v>100</v>
-      </c>
-      <c r="AW6" t="inlineStr">
-        <is>
-          <t>Resource Choice Chest (UR)</t>
-        </is>
-      </c>
-      <c r="AX6" t="n">
-        <v>10</v>
-      </c>
-      <c r="AY6" t="n">
-        <v>50</v>
-      </c>
-      <c r="AZ6" t="inlineStr">
-        <is>
-          <t>BOUN</t>
         </is>
       </c>
       <c r="BA6" t="n">
@@ -1962,94 +2030,113 @@
       </c>
       <c r="BC6" t="inlineStr">
         <is>
+          <t>Resource Choice Chest (UR)</t>
+        </is>
+      </c>
+      <c r="BD6" t="n">
+        <v>10</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>50</v>
+      </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>BOUN</t>
+        </is>
+      </c>
+      <c r="BG6" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI6" t="inlineStr">
+        <is>
           <t>Dual Propeller Base</t>
         </is>
       </c>
-      <c r="BD6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE6" t="n">
+      <c r="BJ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK6" t="n">
         <v>4000</v>
       </c>
-      <c r="BF6" t="inlineStr">
+      <c r="BL6" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI6" t="inlineStr">
+      <c r="BM6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO6" t="inlineStr">
         <is>
           <t>Lv 5 Drone Component Chest</t>
         </is>
       </c>
-      <c r="BJ6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK6" t="n">
+      <c r="BP6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ6" t="n">
         <v>30</v>
       </c>
-      <c r="BL6" t="inlineStr">
+      <c r="BR6" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM6" t="n">
+      <c r="BS6" t="n">
         <v>50</v>
       </c>
-      <c r="BO6" t="inlineStr">
+      <c r="BU6" t="inlineStr">
         <is>
           <t>Iron Chest (SSR)</t>
         </is>
       </c>
-      <c r="BP6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ6" t="n">
+      <c r="BV6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW6" t="n">
         <v>20</v>
       </c>
-      <c r="BR6" t="inlineStr">
+      <c r="BX6" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS6" t="n">
-        <v>10</v>
-      </c>
-      <c r="CA6" t="inlineStr">
+      <c r="BY6" t="n">
+        <v>10</v>
+      </c>
+      <c r="CG6" t="inlineStr">
         <is>
           <t>Universal Exclusive Weapon Shard</t>
         </is>
       </c>
-      <c r="CB6" t="n">
-        <v>10</v>
-      </c>
-      <c r="CC6" t="n">
+      <c r="CH6" t="n">
+        <v>10</v>
+      </c>
+      <c r="CI6" t="n">
         <v>100</v>
       </c>
-      <c r="CD6" t="inlineStr">
+      <c r="CJ6" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CG6" t="inlineStr">
+      <c r="CM6" t="inlineStr">
         <is>
           <t>S1 Skill Point</t>
         </is>
       </c>
-      <c r="CH6" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI6" t="n">
+      <c r="CN6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO6" t="n">
         <v>50</v>
       </c>
-      <c r="CJ6" t="inlineStr">
+      <c r="CP6" t="inlineStr">
         <is>
           <t>SEA</t>
         </is>
       </c>
-      <c r="CK6" t="n">
+      <c r="CQ6" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2184,39 +2271,20 @@
       <c r="AO7" t="n">
         <v>1</v>
       </c>
-      <c r="AQ7" t="inlineStr">
+      <c r="AW7" t="inlineStr">
         <is>
           <t>Valor Badge</t>
         </is>
       </c>
-      <c r="AR7" t="n">
-        <v>10</v>
-      </c>
-      <c r="AS7" t="n">
+      <c r="AX7" t="n">
+        <v>10</v>
+      </c>
+      <c r="AY7" t="n">
         <v>200</v>
       </c>
-      <c r="AT7" t="inlineStr">
+      <c r="AZ7" t="inlineStr">
         <is>
           <t>COUR</t>
-        </is>
-      </c>
-      <c r="AU7" t="n">
-        <v>50</v>
-      </c>
-      <c r="AW7" t="inlineStr">
-        <is>
-          <t>1h Universal Speed-Up</t>
-        </is>
-      </c>
-      <c r="AX7" t="n">
-        <v>10</v>
-      </c>
-      <c r="AY7" t="n">
-        <v>20</v>
-      </c>
-      <c r="AZ7" t="inlineStr">
-        <is>
-          <t>BOUN</t>
         </is>
       </c>
       <c r="BA7" t="n">
@@ -2224,97 +2292,116 @@
       </c>
       <c r="BC7" t="inlineStr">
         <is>
+          <t>1h Universal Speed-Up</t>
+        </is>
+      </c>
+      <c r="BD7" t="n">
+        <v>10</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>20</v>
+      </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>BOUN</t>
+        </is>
+      </c>
+      <c r="BG7" t="n">
+        <v>50</v>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
           <t>Tower of Victory (UR Deco)</t>
         </is>
       </c>
-      <c r="BD7" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE7" t="n">
+      <c r="BJ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK7" t="n">
         <v>100</v>
       </c>
-      <c r="BF7" t="inlineStr">
+      <c r="BL7" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG7" t="n">
+      <c r="BM7" t="n">
         <v>81</v>
       </c>
-      <c r="BI7" t="inlineStr">
+      <c r="BO7" t="inlineStr">
         <is>
           <t>UR Gear Blueprint</t>
         </is>
       </c>
-      <c r="BJ7" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK7" t="n">
+      <c r="BP7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ7" t="n">
         <v>12</v>
       </c>
-      <c r="BL7" t="inlineStr">
+      <c r="BR7" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM7" t="n">
+      <c r="BS7" t="n">
         <v>12</v>
       </c>
-      <c r="BO7" t="inlineStr">
+      <c r="BU7" t="inlineStr">
         <is>
           <t>Food Chest (SSR)</t>
         </is>
       </c>
-      <c r="BP7" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ7" t="n">
+      <c r="BV7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW7" t="n">
         <v>20</v>
       </c>
-      <c r="BR7" t="inlineStr">
+      <c r="BX7" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS7" t="n">
-        <v>10</v>
-      </c>
-      <c r="CA7" t="inlineStr">
+      <c r="BY7" t="n">
+        <v>10</v>
+      </c>
+      <c r="CG7" t="inlineStr">
         <is>
           <t>Recruitment Orders</t>
         </is>
       </c>
-      <c r="CB7" t="n">
+      <c r="CH7" t="n">
         <v>1000</v>
       </c>
-      <c r="CC7" t="n">
+      <c r="CI7" t="n">
         <v>500</v>
       </c>
-      <c r="CD7" t="inlineStr">
+      <c r="CJ7" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE7" t="n">
-        <v>1</v>
-      </c>
-      <c r="CG7" t="inlineStr">
+      <c r="CK7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM7" t="inlineStr">
         <is>
           <t>Profession Change Certificate</t>
         </is>
       </c>
-      <c r="CH7" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI7" t="n">
+      <c r="CN7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO7" t="n">
         <v>50</v>
       </c>
-      <c r="CJ7" t="inlineStr">
+      <c r="CP7" t="inlineStr">
         <is>
           <t>SEA</t>
         </is>
       </c>
-      <c r="CK7" t="n">
+      <c r="CQ7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2411,137 +2498,137 @@
       <c r="AC8" t="n">
         <v>1</v>
       </c>
-      <c r="AQ8" t="inlineStr">
+      <c r="AW8" t="inlineStr">
         <is>
           <t>Drone Parts</t>
         </is>
       </c>
-      <c r="AR8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS8" t="n">
+      <c r="AX8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY8" t="n">
         <v>200</v>
       </c>
-      <c r="AT8" t="inlineStr">
+      <c r="AZ8" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU8" t="n">
+      <c r="BA8" t="n">
         <v>50</v>
       </c>
-      <c r="AW8" t="inlineStr">
+      <c r="BC8" t="inlineStr">
         <is>
           <t>Decoration Chest (UR)</t>
         </is>
       </c>
-      <c r="AX8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY8" t="n">
+      <c r="BD8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE8" t="n">
         <v>100</v>
       </c>
-      <c r="AZ8" t="inlineStr">
+      <c r="BF8" t="inlineStr">
         <is>
           <t>BOUN</t>
         </is>
       </c>
-      <c r="BA8" t="n">
+      <c r="BG8" t="n">
         <v>30</v>
       </c>
-      <c r="BC8" t="inlineStr">
+      <c r="BI8" t="inlineStr">
         <is>
           <t>Gear Blueprint (MR)</t>
         </is>
       </c>
-      <c r="BD8" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE8" t="n">
+      <c r="BJ8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK8" t="n">
         <v>300</v>
       </c>
-      <c r="BF8" t="inlineStr">
+      <c r="BL8" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG8" t="n">
-        <v>10</v>
-      </c>
-      <c r="BI8" t="inlineStr">
+      <c r="BM8" t="n">
+        <v>10</v>
+      </c>
+      <c r="BO8" t="inlineStr">
         <is>
           <t>Premium Chip Material</t>
         </is>
       </c>
-      <c r="BJ8" t="n">
+      <c r="BP8" t="n">
         <v>100</v>
       </c>
-      <c r="BK8" t="n">
+      <c r="BQ8" t="n">
         <v>7</v>
       </c>
-      <c r="BL8" t="inlineStr">
+      <c r="BR8" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM8" t="n">
+      <c r="BS8" t="n">
         <v>80</v>
       </c>
-      <c r="BO8" t="inlineStr">
+      <c r="BU8" t="inlineStr">
         <is>
           <t>Coin Chest (SSR)</t>
         </is>
       </c>
-      <c r="BP8" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ8" t="n">
+      <c r="BV8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW8" t="n">
         <v>20</v>
       </c>
-      <c r="BR8" t="inlineStr">
+      <c r="BX8" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS8" t="n">
-        <v>10</v>
-      </c>
-      <c r="CA8" t="inlineStr">
+      <c r="BY8" t="n">
+        <v>10</v>
+      </c>
+      <c r="CG8" t="inlineStr">
         <is>
           <t>Profession EXP</t>
         </is>
       </c>
-      <c r="CB8" t="n">
+      <c r="CH8" t="n">
         <v>10000</v>
       </c>
-      <c r="CC8" t="n">
+      <c r="CI8" t="n">
         <v>20</v>
       </c>
-      <c r="CD8" t="inlineStr">
+      <c r="CJ8" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE8" t="n">
+      <c r="CK8" t="n">
         <v>20</v>
       </c>
-      <c r="CG8" t="inlineStr">
+      <c r="CM8" t="inlineStr">
         <is>
           <t>Profession Skill Reset Book</t>
         </is>
       </c>
-      <c r="CH8" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI8" t="n">
-        <v>10</v>
-      </c>
-      <c r="CJ8" t="inlineStr">
+      <c r="CN8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO8" t="n">
+        <v>10</v>
+      </c>
+      <c r="CP8" t="inlineStr">
         <is>
           <t>SEA</t>
         </is>
       </c>
-      <c r="CK8" t="n">
+      <c r="CQ8" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2638,77 +2725,58 @@
       <c r="AC9" t="n">
         <v>1</v>
       </c>
-      <c r="AQ9" t="inlineStr">
+      <c r="AW9" t="inlineStr">
         <is>
           <t>Synthetic Resin</t>
         </is>
       </c>
-      <c r="AR9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS9" t="n">
+      <c r="AX9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY9" t="n">
         <v>8</v>
       </c>
-      <c r="AT9" t="inlineStr">
+      <c r="AZ9" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU9" t="n">
+      <c r="BA9" t="n">
         <v>300</v>
       </c>
-      <c r="AW9" t="inlineStr">
+      <c r="BC9" t="inlineStr">
         <is>
           <t>Battle Data (10k)</t>
         </is>
       </c>
-      <c r="AX9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY9" t="n">
+      <c r="BD9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE9" t="n">
         <v>20</v>
       </c>
-      <c r="AZ9" t="inlineStr">
+      <c r="BF9" t="inlineStr">
         <is>
           <t>BOUN</t>
         </is>
       </c>
-      <c r="BA9" t="n">
+      <c r="BG9" t="n">
         <v>200</v>
       </c>
-      <c r="BC9" t="inlineStr">
+      <c r="BI9" t="inlineStr">
         <is>
           <t>UR Hero Universal Shard</t>
         </is>
       </c>
-      <c r="BD9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE9" t="n">
-        <v>10</v>
-      </c>
-      <c r="BF9" t="inlineStr">
+      <c r="BJ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL9" t="inlineStr">
         <is>
           <t>GLIT</t>
-        </is>
-      </c>
-      <c r="BG9" t="n">
-        <v>300</v>
-      </c>
-      <c r="BI9" t="inlineStr">
-        <is>
-          <t>Hero EXP Chest (SSR)</t>
-        </is>
-      </c>
-      <c r="BJ9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL9" t="inlineStr">
-        <is>
-          <t>MOB</t>
         </is>
       </c>
       <c r="BM9" t="n">
@@ -2716,59 +2784,78 @@
       </c>
       <c r="BO9" t="inlineStr">
         <is>
+          <t>Hero EXP Chest (SSR)</t>
+        </is>
+      </c>
+      <c r="BP9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR9" t="inlineStr">
+        <is>
+          <t>MOB</t>
+        </is>
+      </c>
+      <c r="BS9" t="n">
+        <v>300</v>
+      </c>
+      <c r="BU9" t="inlineStr">
+        <is>
           <t>Drone Parts</t>
         </is>
       </c>
-      <c r="BP9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ9" t="n">
+      <c r="BV9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW9" t="n">
         <v>20</v>
       </c>
-      <c r="BR9" t="inlineStr">
+      <c r="BX9" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS9" t="n">
-        <v>10</v>
-      </c>
-      <c r="CA9" t="inlineStr">
+      <c r="BY9" t="n">
+        <v>10</v>
+      </c>
+      <c r="CG9" t="inlineStr">
         <is>
           <t>Mutant Crystals</t>
         </is>
       </c>
-      <c r="CB9" t="n">
+      <c r="CH9" t="n">
         <v>10000</v>
       </c>
-      <c r="CC9" t="n">
-        <v>10</v>
-      </c>
-      <c r="CD9" t="inlineStr">
+      <c r="CI9" t="n">
+        <v>10</v>
+      </c>
+      <c r="CJ9" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE9" t="n">
+      <c r="CK9" t="n">
         <v>50</v>
       </c>
-      <c r="CG9" t="inlineStr">
+      <c r="CM9" t="inlineStr">
         <is>
           <t>Sandstorm Master (Permanent)</t>
         </is>
       </c>
-      <c r="CH9" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI9" t="n">
+      <c r="CN9" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO9" t="n">
         <v>200</v>
       </c>
-      <c r="CJ9" t="inlineStr">
+      <c r="CP9" t="inlineStr">
         <is>
           <t>SEA</t>
         </is>
       </c>
-      <c r="CK9" t="n">
+      <c r="CQ9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2865,137 +2952,137 @@
       <c r="AC10" t="n">
         <v>20</v>
       </c>
-      <c r="AQ10" t="inlineStr">
+      <c r="AW10" t="inlineStr">
         <is>
           <t>Upgrade Ore</t>
         </is>
       </c>
-      <c r="AR10" t="n">
+      <c r="AX10" t="n">
         <v>50</v>
       </c>
-      <c r="AS10" t="n">
+      <c r="AY10" t="n">
         <v>100</v>
       </c>
-      <c r="AT10" t="inlineStr">
+      <c r="AZ10" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU10" t="n">
+      <c r="BA10" t="n">
         <v>100</v>
       </c>
-      <c r="AW10" t="inlineStr">
+      <c r="BC10" t="inlineStr">
         <is>
           <t>UR Hero Universal Shard</t>
         </is>
       </c>
-      <c r="AX10" t="n">
-        <v>10</v>
-      </c>
-      <c r="AY10" t="n">
+      <c r="BD10" t="n">
+        <v>10</v>
+      </c>
+      <c r="BE10" t="n">
         <v>80</v>
       </c>
-      <c r="AZ10" t="inlineStr">
+      <c r="BF10" t="inlineStr">
         <is>
           <t>BOUN</t>
         </is>
       </c>
-      <c r="BA10" t="n">
+      <c r="BG10" t="n">
         <v>20</v>
       </c>
-      <c r="BC10" t="inlineStr">
+      <c r="BI10" t="inlineStr">
         <is>
           <t>Hero EXP Chest (SSR)</t>
         </is>
       </c>
-      <c r="BD10" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE10" t="n">
+      <c r="BJ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK10" t="n">
         <v>6</v>
       </c>
-      <c r="BF10" t="inlineStr">
+      <c r="BL10" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG10" t="n">
+      <c r="BM10" t="n">
         <v>300</v>
       </c>
-      <c r="BI10" t="inlineStr">
+      <c r="BO10" t="inlineStr">
         <is>
           <t>Upgrade Ore</t>
         </is>
       </c>
-      <c r="BJ10" t="n">
+      <c r="BP10" t="n">
         <v>120</v>
       </c>
-      <c r="BK10" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL10" t="inlineStr">
+      <c r="BQ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR10" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM10" t="n">
+      <c r="BS10" t="n">
         <v>1000</v>
       </c>
-      <c r="BO10" t="inlineStr">
+      <c r="BU10" t="inlineStr">
         <is>
           <t>1h Construction Speed-Up</t>
         </is>
       </c>
-      <c r="BP10" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ10" t="n">
-        <v>10</v>
-      </c>
-      <c r="BR10" t="inlineStr">
+      <c r="BV10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>10</v>
+      </c>
+      <c r="BX10" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS10" t="n">
-        <v>10</v>
-      </c>
-      <c r="CA10" t="inlineStr">
+      <c r="BY10" t="n">
+        <v>10</v>
+      </c>
+      <c r="CG10" t="inlineStr">
         <is>
           <t>Iron Chest (SSR)</t>
         </is>
       </c>
-      <c r="CB10" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC10" t="n">
+      <c r="CH10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI10" t="n">
         <v>20</v>
       </c>
-      <c r="CD10" t="inlineStr">
+      <c r="CJ10" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE10" t="n">
+      <c r="CK10" t="n">
         <v>100</v>
       </c>
-      <c r="CG10" t="inlineStr">
+      <c r="CM10" t="inlineStr">
         <is>
           <t>UR Hero Badge</t>
         </is>
       </c>
-      <c r="CH10" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI10" t="n">
+      <c r="CN10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO10" t="n">
         <v>50</v>
       </c>
-      <c r="CJ10" t="inlineStr">
+      <c r="CP10" t="inlineStr">
         <is>
           <t>SEA</t>
         </is>
       </c>
-      <c r="CK10" t="n">
+      <c r="CQ10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3076,43 +3163,24 @@
       <c r="AC11" t="n">
         <v>10</v>
       </c>
-      <c r="AQ11" t="inlineStr">
+      <c r="AW11" t="inlineStr">
         <is>
           <t>Hero Recruitment Ticket</t>
         </is>
       </c>
-      <c r="AR11" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS11" t="n">
+      <c r="AX11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY11" t="n">
         <v>80</v>
       </c>
-      <c r="AT11" t="inlineStr">
+      <c r="AZ11" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU11" t="n">
-        <v>10</v>
-      </c>
-      <c r="AW11" t="inlineStr">
-        <is>
-          <t>Skill Medal</t>
-        </is>
-      </c>
-      <c r="AX11" t="n">
-        <v>1000</v>
-      </c>
-      <c r="AY11" t="n">
-        <v>15</v>
-      </c>
-      <c r="AZ11" t="inlineStr">
-        <is>
-          <t>BOUN</t>
-        </is>
-      </c>
       <c r="BA11" t="n">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="BC11" t="inlineStr">
         <is>
@@ -3127,67 +3195,86 @@
       </c>
       <c r="BF11" t="inlineStr">
         <is>
+          <t>BOUN</t>
+        </is>
+      </c>
+      <c r="BG11" t="n">
+        <v>150</v>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>Skill Medal</t>
+        </is>
+      </c>
+      <c r="BJ11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>15</v>
+      </c>
+      <c r="BL11" t="inlineStr">
+        <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG11" t="n">
+      <c r="BM11" t="n">
         <v>300</v>
       </c>
-      <c r="BI11" t="inlineStr">
+      <c r="BO11" t="inlineStr">
         <is>
           <t>Skill Medal</t>
         </is>
       </c>
-      <c r="BJ11" t="n">
+      <c r="BP11" t="n">
         <v>200</v>
       </c>
-      <c r="BK11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL11" t="inlineStr">
+      <c r="BQ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR11" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM11" t="n">
+      <c r="BS11" t="n">
         <v>1000</v>
       </c>
-      <c r="BO11" t="inlineStr">
+      <c r="BU11" t="inlineStr">
         <is>
           <t>1h Research Speed-Up</t>
         </is>
       </c>
-      <c r="BP11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ11" t="n">
-        <v>10</v>
-      </c>
-      <c r="BR11" t="inlineStr">
+      <c r="BV11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>10</v>
+      </c>
+      <c r="BX11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS11" t="n">
-        <v>10</v>
-      </c>
-      <c r="CA11" t="inlineStr">
+      <c r="BY11" t="n">
+        <v>10</v>
+      </c>
+      <c r="CG11" t="inlineStr">
         <is>
           <t>Coin Chest (SSR)</t>
         </is>
       </c>
-      <c r="CB11" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC11" t="n">
+      <c r="CH11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI11" t="n">
         <v>20</v>
       </c>
-      <c r="CD11" t="inlineStr">
+      <c r="CJ11" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE11" t="n">
+      <c r="CK11" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3268,118 +3355,118 @@
       <c r="AC12" t="n">
         <v>30</v>
       </c>
-      <c r="AQ12" t="inlineStr">
+      <c r="AW12" t="inlineStr">
         <is>
           <t>Stamina</t>
         </is>
       </c>
-      <c r="AR12" t="n">
+      <c r="AX12" t="n">
         <v>50</v>
       </c>
-      <c r="AS12" t="n">
-        <v>10</v>
-      </c>
-      <c r="AT12" t="inlineStr">
+      <c r="AY12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AZ12" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU12" t="n">
+      <c r="BA12" t="n">
         <v>3</v>
       </c>
-      <c r="AW12" t="inlineStr">
+      <c r="BC12" t="inlineStr">
         <is>
           <t>Drone Parts</t>
         </is>
       </c>
-      <c r="AX12" t="n">
-        <v>10</v>
-      </c>
-      <c r="AY12" t="n">
+      <c r="BD12" t="n">
+        <v>10</v>
+      </c>
+      <c r="BE12" t="n">
         <v>32</v>
       </c>
-      <c r="AZ12" t="inlineStr">
+      <c r="BF12" t="inlineStr">
         <is>
           <t>BOUN</t>
         </is>
       </c>
-      <c r="BA12" t="n">
+      <c r="BG12" t="n">
         <v>300</v>
       </c>
-      <c r="BC12" t="inlineStr">
+      <c r="BI12" t="inlineStr">
         <is>
           <t>Valor Badge</t>
         </is>
       </c>
-      <c r="BD12" t="n">
+      <c r="BJ12" t="n">
         <v>100</v>
       </c>
-      <c r="BE12" t="n">
+      <c r="BK12" t="n">
         <v>50</v>
       </c>
-      <c r="BF12" t="inlineStr">
+      <c r="BL12" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG12" t="n">
+      <c r="BM12" t="n">
         <v>200</v>
       </c>
-      <c r="BI12" t="inlineStr">
+      <c r="BO12" t="inlineStr">
         <is>
           <t>Resource Choice Chest (SSR)</t>
         </is>
       </c>
-      <c r="BJ12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL12" t="inlineStr">
+      <c r="BP12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR12" t="inlineStr">
         <is>
           <t>MOB</t>
         </is>
       </c>
-      <c r="BM12" t="n">
+      <c r="BS12" t="n">
         <v>4000</v>
       </c>
-      <c r="BO12" t="inlineStr">
+      <c r="BU12" t="inlineStr">
         <is>
           <t>1h Training Speed-Up</t>
         </is>
       </c>
-      <c r="BP12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ12" t="n">
-        <v>10</v>
-      </c>
-      <c r="BR12" t="inlineStr">
+      <c r="BV12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>10</v>
+      </c>
+      <c r="BX12" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS12" t="n">
-        <v>10</v>
-      </c>
-      <c r="CA12" t="inlineStr">
+      <c r="BY12" t="n">
+        <v>10</v>
+      </c>
+      <c r="CG12" t="inlineStr">
         <is>
           <t>Food Chest (SSR)</t>
         </is>
       </c>
-      <c r="CB12" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC12" t="n">
+      <c r="CH12" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI12" t="n">
         <v>20</v>
       </c>
-      <c r="CD12" t="inlineStr">
+      <c r="CJ12" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE12" t="n">
+      <c r="CK12" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3460,99 +3547,99 @@
       <c r="AC13" t="n">
         <v>30</v>
       </c>
-      <c r="AQ13" t="inlineStr">
+      <c r="AW13" t="inlineStr">
         <is>
           <t>Lv 3 Drone Component Chest</t>
         </is>
       </c>
-      <c r="AR13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS13" t="n">
+      <c r="AX13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY13" t="n">
         <v>360</v>
       </c>
-      <c r="AT13" t="inlineStr">
+      <c r="AZ13" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU13" t="n">
+      <c r="BA13" t="n">
         <v>3</v>
       </c>
-      <c r="AW13" t="inlineStr">
+      <c r="BC13" t="inlineStr">
         <is>
           <t>Valor Badge</t>
         </is>
       </c>
-      <c r="AX13" t="n">
+      <c r="BD13" t="n">
         <v>100</v>
       </c>
-      <c r="AY13" t="n">
+      <c r="BE13" t="n">
         <v>50</v>
       </c>
-      <c r="AZ13" t="inlineStr">
+      <c r="BF13" t="inlineStr">
         <is>
           <t>BOUN</t>
         </is>
       </c>
-      <c r="BA13" t="n">
+      <c r="BG13" t="n">
         <v>100</v>
       </c>
-      <c r="BC13" t="inlineStr">
+      <c r="BI13" t="inlineStr">
         <is>
           <t>1h Universal Speed-Up</t>
         </is>
       </c>
-      <c r="BD13" t="n">
-        <v>10</v>
-      </c>
-      <c r="BE13" t="n">
+      <c r="BJ13" t="n">
+        <v>10</v>
+      </c>
+      <c r="BK13" t="n">
         <v>25</v>
       </c>
-      <c r="BF13" t="inlineStr">
+      <c r="BL13" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG13" t="n">
+      <c r="BM13" t="n">
         <v>200</v>
       </c>
-      <c r="BO13" t="inlineStr">
+      <c r="BU13" t="inlineStr">
         <is>
           <t>1h Healing Speed-Up</t>
         </is>
       </c>
-      <c r="BP13" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ13" t="n">
-        <v>10</v>
-      </c>
-      <c r="BR13" t="inlineStr">
+      <c r="BV13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>10</v>
+      </c>
+      <c r="BX13" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="BS13" t="n">
-        <v>10</v>
-      </c>
-      <c r="CA13" t="inlineStr">
+      <c r="BY13" t="n">
+        <v>10</v>
+      </c>
+      <c r="CG13" t="inlineStr">
         <is>
           <t>5m Construction Speed-Up</t>
         </is>
       </c>
-      <c r="CB13" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC13" t="n">
-        <v>1</v>
-      </c>
-      <c r="CD13" t="inlineStr">
+      <c r="CH13" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI13" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ13" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE13" t="n">
+      <c r="CK13" t="n">
         <v>9999</v>
       </c>
     </row>
@@ -3614,61 +3701,61 @@
       <c r="AC14" t="n">
         <v>100</v>
       </c>
-      <c r="AQ14" t="inlineStr">
+      <c r="AW14" t="inlineStr">
         <is>
           <t>5m Research Speed-Up</t>
         </is>
       </c>
-      <c r="AR14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS14" t="n">
+      <c r="AX14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY14" t="n">
         <v>4</v>
       </c>
-      <c r="AT14" t="inlineStr">
+      <c r="AZ14" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU14" t="n">
+      <c r="BA14" t="n">
         <v>100</v>
       </c>
-      <c r="BC14" t="inlineStr">
+      <c r="BI14" t="inlineStr">
         <is>
           <t>Resource Choice Chest (SSR)</t>
         </is>
       </c>
-      <c r="BD14" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE14" t="n">
+      <c r="BJ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK14" t="n">
         <v>2</v>
       </c>
-      <c r="BF14" t="inlineStr">
+      <c r="BL14" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG14" t="n">
+      <c r="BM14" t="n">
         <v>1000</v>
       </c>
-      <c r="CA14" t="inlineStr">
+      <c r="CG14" t="inlineStr">
         <is>
           <t>5m Research Speed-Up</t>
         </is>
       </c>
-      <c r="CB14" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC14" t="n">
-        <v>1</v>
-      </c>
-      <c r="CD14" t="inlineStr">
+      <c r="CH14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ14" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE14" t="n">
+      <c r="CK14" t="n">
         <v>9999</v>
       </c>
     </row>
@@ -3730,61 +3817,61 @@
       <c r="AC15" t="n">
         <v>200</v>
       </c>
-      <c r="AQ15" t="inlineStr">
+      <c r="AW15" t="inlineStr">
         <is>
           <t>5m Construction Speed-Up</t>
         </is>
       </c>
-      <c r="AR15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS15" t="n">
+      <c r="AX15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY15" t="n">
         <v>4</v>
       </c>
-      <c r="AT15" t="inlineStr">
+      <c r="AZ15" t="inlineStr">
         <is>
           <t>COUR</t>
         </is>
       </c>
-      <c r="AU15" t="n">
+      <c r="BA15" t="n">
         <v>50</v>
       </c>
-      <c r="BC15" t="inlineStr">
+      <c r="BI15" t="inlineStr">
         <is>
           <t>Dielectric Ceramic</t>
         </is>
       </c>
-      <c r="BD15" t="n">
+      <c r="BJ15" t="n">
         <v>100</v>
       </c>
-      <c r="BE15" t="n">
+      <c r="BK15" t="n">
         <v>60</v>
       </c>
-      <c r="BF15" t="inlineStr">
+      <c r="BL15" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG15" t="n">
+      <c r="BM15" t="n">
         <v>200</v>
       </c>
-      <c r="CA15" t="inlineStr">
+      <c r="CG15" t="inlineStr">
         <is>
           <t>5m Training Speed-Up</t>
         </is>
       </c>
-      <c r="CB15" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC15" t="n">
-        <v>1</v>
-      </c>
-      <c r="CD15" t="inlineStr">
+      <c r="CH15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ15" t="inlineStr">
         <is>
           <t>SER</t>
         </is>
       </c>
-      <c r="CE15" t="n">
+      <c r="CK15" t="n">
         <v>9999</v>
       </c>
     </row>
@@ -3846,23 +3933,23 @@
       <c r="AC16" t="n">
         <v>750</v>
       </c>
-      <c r="BC16" t="inlineStr">
+      <c r="BI16" t="inlineStr">
         <is>
           <t>Upgrade Ore</t>
         </is>
       </c>
-      <c r="BD16" t="n">
+      <c r="BJ16" t="n">
         <v>10000</v>
       </c>
-      <c r="BE16" t="n">
+      <c r="BK16" t="n">
         <v>250</v>
       </c>
-      <c r="BF16" t="inlineStr">
+      <c r="BL16" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG16" t="n">
+      <c r="BM16" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3924,23 +4011,23 @@
       <c r="AC17" t="n">
         <v>200</v>
       </c>
-      <c r="BC17" t="inlineStr">
+      <c r="BI17" t="inlineStr">
         <is>
           <t>Gear Blueprint (UR)</t>
         </is>
       </c>
-      <c r="BD17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE17" t="n">
+      <c r="BJ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK17" t="n">
         <v>60</v>
       </c>
-      <c r="BF17" t="inlineStr">
+      <c r="BL17" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG17" t="n">
+      <c r="BM17" t="n">
         <v>150</v>
       </c>
     </row>
@@ -4002,23 +4089,23 @@
       <c r="AC18" t="n">
         <v>200</v>
       </c>
-      <c r="BC18" t="inlineStr">
+      <c r="BI18" t="inlineStr">
         <is>
           <t>Training Tire (SSR Deco)</t>
         </is>
       </c>
-      <c r="BD18" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE18" t="n">
+      <c r="BJ18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK18" t="n">
         <v>40</v>
       </c>
-      <c r="BF18" t="inlineStr">
+      <c r="BL18" t="inlineStr">
         <is>
           <t>GLIT</t>
         </is>
       </c>
-      <c r="BG18" t="n">
+      <c r="BM18" t="n">
         <v>81</v>
       </c>
     </row>

</xml_diff>